<commit_message>
Remove old Swift app source and reorganized example files
The Swift app files under ELISAWorkflowApp/ and the original
Example Input/ CSVs were superseded in the previous commit but
not removed from tracking. Also removes the old README, SOP PDF,
and manually written notebook that no longer belong at top level.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Example/ELISA_Output.xlsx
+++ b/Example/ELISA_Output.xlsx
@@ -65,12 +65,48 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.7999816888943144"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.5999938962981048"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.09997863704336681"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.5999938962981048"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.7999816888943144"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -97,12 +133,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -113,10 +155,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -871,57 +913,39 @@
           <t>blank</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>sample 1</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>sample 2</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>sample 3</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>sample 4</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>sample 5</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>sample 6</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>sample 7</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>sample 8</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>sample 9</t>
-        </is>
+      <c r="C8" s="1" t="n">
+        <v>64</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>92</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>201</v>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>203</v>
+      </c>
+      <c r="G8" s="1" t="n">
+        <v>276</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>199</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>202</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>206</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>299</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>sample 10</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
+          <t>blank</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
@@ -931,57 +955,39 @@
           <t>blank</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>sample 1</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>sample 2</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>sample 3</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>sample 4</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>sample 5</t>
-        </is>
-      </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>sample 6</t>
-        </is>
-      </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>sample 7</t>
-        </is>
-      </c>
-      <c r="X8" t="inlineStr">
-        <is>
-          <t>sample 8</t>
-        </is>
-      </c>
-      <c r="Y8" t="inlineStr">
-        <is>
-          <t>sample 9</t>
-        </is>
+      <c r="Q8" s="2" t="n">
+        <v>989</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>171</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>172</v>
+      </c>
+      <c r="T8" s="4" t="n">
+        <v>173</v>
+      </c>
+      <c r="U8" s="4" t="n">
+        <v>204</v>
+      </c>
+      <c r="V8" s="4" t="n">
+        <v>210</v>
+      </c>
+      <c r="W8" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="X8" s="5" t="n">
+        <v>51</v>
+      </c>
+      <c r="Y8" s="5" t="n">
+        <v>52</v>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>sample 10</t>
-        </is>
-      </c>
-      <c r="AA8" t="inlineStr">
+          <t>blank</t>
+        </is>
+      </c>
+      <c r="AA8" s="3" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
@@ -991,57 +997,43 @@
           <t>blank</t>
         </is>
       </c>
-      <c r="AE8" t="inlineStr">
-        <is>
-          <t>sample 1</t>
-        </is>
-      </c>
-      <c r="AF8" t="inlineStr">
-        <is>
-          <t>sample 2</t>
-        </is>
-      </c>
-      <c r="AG8" t="inlineStr">
-        <is>
-          <t>sample 3</t>
-        </is>
-      </c>
-      <c r="AH8" t="inlineStr">
-        <is>
-          <t>sample 4</t>
-        </is>
-      </c>
-      <c r="AI8" t="inlineStr">
-        <is>
-          <t>sample 5</t>
-        </is>
-      </c>
-      <c r="AJ8" t="inlineStr">
-        <is>
-          <t>sample 6</t>
-        </is>
-      </c>
-      <c r="AK8" t="inlineStr">
-        <is>
-          <t>sample 7</t>
-        </is>
+      <c r="AE8" s="5" t="n">
+        <v>238</v>
+      </c>
+      <c r="AF8" s="5" t="n">
+        <v>264</v>
+      </c>
+      <c r="AG8" s="6" t="n">
+        <v>693</v>
+      </c>
+      <c r="AH8" s="6" t="n">
+        <v>694</v>
+      </c>
+      <c r="AI8" s="6" t="n">
+        <v>695</v>
+      </c>
+      <c r="AJ8" s="6" t="n">
+        <v>696</v>
+      </c>
+      <c r="AK8" s="6" t="n">
+        <v>697</v>
       </c>
       <c r="AL8" t="inlineStr">
         <is>
-          <t>sample 8</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="AM8" t="inlineStr">
         <is>
-          <t>sample 9</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="AN8" t="inlineStr">
         <is>
-          <t>sample 10</t>
-        </is>
-      </c>
-      <c r="AO8" t="inlineStr">
+          <t>blank</t>
+        </is>
+      </c>
+      <c r="AO8" s="3" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
@@ -1051,57 +1043,39 @@
           <t>blank</t>
         </is>
       </c>
-      <c r="AS8" t="inlineStr">
-        <is>
-          <t>sample 1</t>
-        </is>
-      </c>
-      <c r="AT8" t="inlineStr">
-        <is>
-          <t>sample 2</t>
-        </is>
-      </c>
-      <c r="AU8" t="inlineStr">
-        <is>
-          <t>sample 3</t>
-        </is>
-      </c>
-      <c r="AV8" t="inlineStr">
-        <is>
-          <t>sample 4</t>
-        </is>
-      </c>
-      <c r="AW8" t="inlineStr">
-        <is>
-          <t>sample 5</t>
-        </is>
-      </c>
-      <c r="AX8" t="inlineStr">
-        <is>
-          <t>sample 6</t>
-        </is>
-      </c>
-      <c r="AY8" t="inlineStr">
-        <is>
-          <t>sample 7</t>
-        </is>
-      </c>
-      <c r="AZ8" t="inlineStr">
-        <is>
-          <t>sample 8</t>
-        </is>
-      </c>
-      <c r="BA8" t="inlineStr">
-        <is>
-          <t>sample 9</t>
-        </is>
+      <c r="AS8" s="1" t="n">
+        <v>64</v>
+      </c>
+      <c r="AT8" s="1" t="n">
+        <v>92</v>
+      </c>
+      <c r="AU8" s="1" t="n">
+        <v>201</v>
+      </c>
+      <c r="AV8" s="1" t="n">
+        <v>203</v>
+      </c>
+      <c r="AW8" s="1" t="n">
+        <v>276</v>
+      </c>
+      <c r="AX8" s="2" t="n">
+        <v>199</v>
+      </c>
+      <c r="AY8" s="2" t="n">
+        <v>202</v>
+      </c>
+      <c r="AZ8" s="2" t="n">
+        <v>206</v>
+      </c>
+      <c r="BA8" s="2" t="n">
+        <v>299</v>
       </c>
       <c r="BB8" t="inlineStr">
         <is>
-          <t>sample 10</t>
-        </is>
-      </c>
-      <c r="BC8" t="inlineStr">
+          <t>blank</t>
+        </is>
+      </c>
+      <c r="BC8" s="3" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
@@ -1111,57 +1085,39 @@
           <t>blank</t>
         </is>
       </c>
-      <c r="BG8" t="inlineStr">
-        <is>
-          <t>sample 1</t>
-        </is>
-      </c>
-      <c r="BH8" t="inlineStr">
-        <is>
-          <t>sample 2</t>
-        </is>
-      </c>
-      <c r="BI8" t="inlineStr">
-        <is>
-          <t>sample 3</t>
-        </is>
-      </c>
-      <c r="BJ8" t="inlineStr">
-        <is>
-          <t>sample 4</t>
-        </is>
-      </c>
-      <c r="BK8" t="inlineStr">
-        <is>
-          <t>sample 5</t>
-        </is>
-      </c>
-      <c r="BL8" t="inlineStr">
-        <is>
-          <t>sample 6</t>
-        </is>
-      </c>
-      <c r="BM8" t="inlineStr">
-        <is>
-          <t>sample 7</t>
-        </is>
-      </c>
-      <c r="BN8" t="inlineStr">
-        <is>
-          <t>sample 8</t>
-        </is>
-      </c>
-      <c r="BO8" t="inlineStr">
-        <is>
-          <t>sample 9</t>
-        </is>
+      <c r="BG8" s="2" t="n">
+        <v>989</v>
+      </c>
+      <c r="BH8" s="4" t="n">
+        <v>171</v>
+      </c>
+      <c r="BI8" s="4" t="n">
+        <v>172</v>
+      </c>
+      <c r="BJ8" s="4" t="n">
+        <v>173</v>
+      </c>
+      <c r="BK8" s="4" t="n">
+        <v>204</v>
+      </c>
+      <c r="BL8" s="4" t="n">
+        <v>210</v>
+      </c>
+      <c r="BM8" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="BN8" s="5" t="n">
+        <v>51</v>
+      </c>
+      <c r="BO8" s="5" t="n">
+        <v>52</v>
       </c>
       <c r="BP8" t="inlineStr">
         <is>
-          <t>sample 10</t>
-        </is>
-      </c>
-      <c r="BQ8" t="inlineStr">
+          <t>blank</t>
+        </is>
+      </c>
+      <c r="BQ8" s="3" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
@@ -1171,57 +1127,43 @@
           <t>blank</t>
         </is>
       </c>
-      <c r="BU8" t="inlineStr">
-        <is>
-          <t>sample 1</t>
-        </is>
-      </c>
-      <c r="BV8" t="inlineStr">
-        <is>
-          <t>sample 2</t>
-        </is>
-      </c>
-      <c r="BW8" t="inlineStr">
-        <is>
-          <t>sample 3</t>
-        </is>
-      </c>
-      <c r="BX8" t="inlineStr">
-        <is>
-          <t>sample 4</t>
-        </is>
-      </c>
-      <c r="BY8" t="inlineStr">
-        <is>
-          <t>sample 5</t>
-        </is>
-      </c>
-      <c r="BZ8" t="inlineStr">
-        <is>
-          <t>sample 6</t>
-        </is>
-      </c>
-      <c r="CA8" t="inlineStr">
-        <is>
-          <t>sample 7</t>
-        </is>
+      <c r="BU8" s="5" t="n">
+        <v>238</v>
+      </c>
+      <c r="BV8" s="5" t="n">
+        <v>264</v>
+      </c>
+      <c r="BW8" s="6" t="n">
+        <v>693</v>
+      </c>
+      <c r="BX8" s="6" t="n">
+        <v>694</v>
+      </c>
+      <c r="BY8" s="6" t="n">
+        <v>695</v>
+      </c>
+      <c r="BZ8" s="6" t="n">
+        <v>696</v>
+      </c>
+      <c r="CA8" s="6" t="n">
+        <v>697</v>
       </c>
       <c r="CB8" t="inlineStr">
         <is>
-          <t>sample 8</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="CC8" t="inlineStr">
         <is>
-          <t>sample 9</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="CD8" t="inlineStr">
         <is>
-          <t>sample 10</t>
-        </is>
-      </c>
-      <c r="CE8" t="inlineStr">
+          <t>blank</t>
+        </is>
+      </c>
+      <c r="CE8" s="3" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
@@ -5704,34 +5646,36 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>413</v>
+        <v>887</v>
       </c>
       <c r="D31" t="n">
-        <v>352</v>
+        <v>762</v>
       </c>
       <c r="E31" t="n">
-        <v>351</v>
+        <v>740</v>
       </c>
       <c r="F31" t="n">
-        <v>374</v>
+        <v>804</v>
       </c>
       <c r="G31" t="n">
         <v>10</v>
       </c>
       <c r="H31" t="n">
-        <v>299</v>
+        <v>630</v>
       </c>
       <c r="I31" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="J31" t="n">
-        <v>228</v>
+        <v>470</v>
       </c>
       <c r="K31" t="n">
-        <v>22</v>
-      </c>
-      <c r="L31" t="n">
-        <v>10</v>
+        <v>20</v>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
@@ -5758,7 +5702,7 @@
         <v>10</v>
       </c>
       <c r="T31" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="U31" t="n">
         <v>10</v>
@@ -5767,106 +5711,116 @@
         <v>10</v>
       </c>
       <c r="W31" t="n">
-        <v>1050</v>
+        <v>2565</v>
       </c>
       <c r="X31" t="n">
-        <v>1135</v>
+        <v>2906</v>
       </c>
       <c r="Y31" t="n">
-        <v>31</v>
-      </c>
-      <c r="Z31" t="n">
+        <v>28</v>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>Est. ED50</t>
+        </is>
+      </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="AE31" t="n">
+        <v>3919</v>
+      </c>
+      <c r="AF31" t="n">
         <v>10</v>
       </c>
-      <c r="AA31" t="inlineStr">
+      <c r="AG31" t="n">
+        <v>117</v>
+      </c>
+      <c r="AH31" t="n">
+        <v>10905</v>
+      </c>
+      <c r="AI31" t="n">
+        <v>10</v>
+      </c>
+      <c r="AJ31" t="n">
+        <v>66</v>
+      </c>
+      <c r="AK31" t="n">
+        <v>558</v>
+      </c>
+      <c r="AL31" t="inlineStr">
         <is>
           <t>/</t>
         </is>
       </c>
-      <c r="AC31" t="inlineStr">
+      <c r="AM31" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="AN31" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="AO31" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="AQ31" t="inlineStr">
         <is>
           <t>Est. ED50</t>
         </is>
       </c>
-      <c r="AD31" t="inlineStr">
+      <c r="AR31" t="inlineStr">
         <is>
           <t>/</t>
         </is>
       </c>
-      <c r="AE31" t="n">
-        <v>1468</v>
-      </c>
-      <c r="AF31" t="n">
-        <v>14</v>
-      </c>
-      <c r="AG31" t="n">
-        <v>62</v>
-      </c>
-      <c r="AH31" t="n">
-        <v>3453</v>
-      </c>
-      <c r="AI31" t="n">
-        <v>14</v>
-      </c>
-      <c r="AJ31" t="n">
-        <v>63</v>
-      </c>
-      <c r="AK31" t="n">
-        <v>264</v>
-      </c>
-      <c r="AL31" t="n">
+      <c r="AS31" t="n">
+        <v>27874</v>
+      </c>
+      <c r="AT31" t="n">
+        <v>28375</v>
+      </c>
+      <c r="AU31" t="n">
+        <v>27279</v>
+      </c>
+      <c r="AV31" t="n">
+        <v>27312</v>
+      </c>
+      <c r="AW31" t="n">
+        <v>31559</v>
+      </c>
+      <c r="AX31" t="n">
+        <v>610</v>
+      </c>
+      <c r="AY31" t="n">
+        <v>38</v>
+      </c>
+      <c r="AZ31" t="n">
         <v>10</v>
-      </c>
-      <c r="AM31" t="n">
-        <v>10</v>
-      </c>
-      <c r="AN31" t="n">
-        <v>10</v>
-      </c>
-      <c r="AO31" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AQ31" t="inlineStr">
-        <is>
-          <t>Est. ED50</t>
-        </is>
-      </c>
-      <c r="AR31" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AS31" t="n">
-        <v>6936</v>
-      </c>
-      <c r="AT31" t="n">
-        <v>7184</v>
-      </c>
-      <c r="AU31" t="n">
-        <v>6893</v>
-      </c>
-      <c r="AV31" t="n">
-        <v>6903</v>
-      </c>
-      <c r="AW31" t="n">
-        <v>7930</v>
-      </c>
-      <c r="AX31" t="n">
-        <v>287</v>
-      </c>
-      <c r="AY31" t="n">
-        <v>22</v>
-      </c>
-      <c r="AZ31" t="n">
-        <v>13</v>
       </c>
       <c r="BA31" t="n">
         <v>10</v>
       </c>
-      <c r="BB31" t="n">
-        <v>10</v>
+      <c r="BB31" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
       <c r="BC31" t="inlineStr">
         <is>
@@ -5890,28 +5844,30 @@
         <v>17</v>
       </c>
       <c r="BI31" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="BJ31" t="n">
         <v>10</v>
       </c>
       <c r="BK31" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="BL31" t="n">
         <v>10</v>
       </c>
       <c r="BM31" t="n">
-        <v>8233</v>
+        <v>32835</v>
       </c>
       <c r="BN31" t="n">
-        <v>7444</v>
+        <v>29312</v>
       </c>
       <c r="BO31" t="n">
-        <v>7074</v>
-      </c>
-      <c r="BP31" t="n">
-        <v>10</v>
+        <v>27570</v>
+      </c>
+      <c r="BP31" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
       <c r="BQ31" t="inlineStr">
         <is>
@@ -5929,34 +5885,40 @@
         </is>
       </c>
       <c r="BU31" t="n">
-        <v>7589</v>
+        <v>29771</v>
       </c>
       <c r="BV31" t="n">
-        <v>7509</v>
+        <v>29652</v>
       </c>
       <c r="BW31" t="n">
-        <v>6956</v>
+        <v>27192</v>
       </c>
       <c r="BX31" t="n">
-        <v>10577</v>
+        <v>45730</v>
       </c>
       <c r="BY31" t="n">
-        <v>7089</v>
+        <v>28997</v>
       </c>
       <c r="BZ31" t="n">
-        <v>7480</v>
+        <v>29825</v>
       </c>
       <c r="CA31" t="n">
-        <v>7867</v>
-      </c>
-      <c r="CB31" t="n">
-        <v>10</v>
-      </c>
-      <c r="CC31" t="n">
-        <v>10</v>
-      </c>
-      <c r="CD31" t="n">
-        <v>10</v>
+        <v>31696</v>
+      </c>
+      <c r="CB31" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="CC31" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="CD31" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
       <c r="CE31" t="inlineStr">
         <is>
@@ -6002,8 +5964,10 @@
       <c r="K33" t="n">
         <v>0.576</v>
       </c>
-      <c r="L33" t="n">
-        <v>0.211</v>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
       <c r="M33" t="n">
         <v>1.156</v>
@@ -6045,8 +6009,10 @@
       <c r="Y33" t="n">
         <v>0.876</v>
       </c>
-      <c r="Z33" t="n">
-        <v>0.159</v>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
       <c r="AA33" t="n">
         <v>0.652</v>
@@ -6082,14 +6048,20 @@
       <c r="AK33" t="n">
         <v>1.224</v>
       </c>
-      <c r="AL33" t="n">
-        <v>0.138</v>
-      </c>
-      <c r="AM33" t="n">
-        <v>0.126</v>
-      </c>
-      <c r="AN33" t="n">
-        <v>0.102</v>
+      <c r="AL33" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="AM33" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="AN33" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
       <c r="AO33" t="n">
         <v>1.889</v>
@@ -6131,8 +6103,10 @@
       <c r="BA33" t="n">
         <v>0.68</v>
       </c>
-      <c r="BB33" t="n">
-        <v>0.065</v>
+      <c r="BB33" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
       <c r="BC33" t="n">
         <v>0.73</v>
@@ -6174,8 +6148,10 @@
       <c r="BO33" t="n">
         <v>0.39</v>
       </c>
-      <c r="BP33" t="n">
-        <v>0.094</v>
+      <c r="BP33" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
       <c r="BQ33" t="n">
         <v>0.704</v>
@@ -6211,14 +6187,20 @@
       <c r="CA33" t="n">
         <v>0.577</v>
       </c>
-      <c r="CB33" t="n">
-        <v>0.081</v>
-      </c>
-      <c r="CC33" t="n">
-        <v>0.105</v>
-      </c>
-      <c r="CD33" t="n">
-        <v>0.062</v>
+      <c r="CB33" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="CC33" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="CD33" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
       <c r="CE33" t="n">
         <v>0.579</v>
@@ -6236,34 +6218,36 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1350</v>
+        <v>3200</v>
       </c>
       <c r="D34" t="n">
-        <v>1350</v>
+        <v>3200</v>
       </c>
       <c r="E34" t="n">
-        <v>450</v>
+        <v>800</v>
       </c>
       <c r="F34" t="n">
-        <v>1350</v>
+        <v>3200</v>
       </c>
       <c r="G34" t="n">
         <v>50</v>
       </c>
       <c r="H34" t="n">
-        <v>450</v>
+        <v>800</v>
       </c>
       <c r="I34" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="J34" t="n">
-        <v>450</v>
+        <v>800</v>
       </c>
       <c r="K34" t="n">
-        <v>150</v>
-      </c>
-      <c r="L34" t="n">
-        <v>50</v>
+        <v>200</v>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
@@ -6299,16 +6283,18 @@
         <v>50</v>
       </c>
       <c r="W34" t="n">
-        <v>450</v>
+        <v>800</v>
       </c>
       <c r="X34" t="n">
-        <v>1350</v>
+        <v>3200</v>
       </c>
       <c r="Y34" t="n">
-        <v>150</v>
-      </c>
-      <c r="Z34" t="n">
-        <v>50</v>
+        <v>200</v>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
       <c r="AA34" t="inlineStr">
         <is>
@@ -6326,34 +6312,40 @@
         </is>
       </c>
       <c r="AE34" t="n">
-        <v>1350</v>
+        <v>3200</v>
       </c>
       <c r="AF34" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="AG34" t="n">
-        <v>450</v>
+        <v>800</v>
       </c>
       <c r="AH34" t="n">
-        <v>4050</v>
+        <v>12800</v>
       </c>
       <c r="AI34" t="n">
         <v>50</v>
       </c>
       <c r="AJ34" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="AK34" t="n">
-        <v>450</v>
-      </c>
-      <c r="AL34" t="n">
-        <v>50</v>
-      </c>
-      <c r="AM34" t="n">
-        <v>50</v>
-      </c>
-      <c r="AN34" t="n">
-        <v>50</v>
+        <v>800</v>
+      </c>
+      <c r="AL34" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="AM34" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="AN34" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
       <c r="AO34" t="inlineStr">
         <is>
@@ -6371,25 +6363,25 @@
         </is>
       </c>
       <c r="AS34" t="n">
-        <v>12150</v>
+        <v>51200</v>
       </c>
       <c r="AT34" t="n">
-        <v>12150</v>
+        <v>51200</v>
       </c>
       <c r="AU34" t="n">
-        <v>12150</v>
+        <v>51200</v>
       </c>
       <c r="AV34" t="n">
-        <v>12150</v>
+        <v>51200</v>
       </c>
       <c r="AW34" t="n">
-        <v>12150</v>
+        <v>51200</v>
       </c>
       <c r="AX34" t="n">
-        <v>450</v>
+        <v>800</v>
       </c>
       <c r="AY34" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="AZ34" t="n">
         <v>50</v>
@@ -6397,8 +6389,10 @@
       <c r="BA34" t="n">
         <v>50</v>
       </c>
-      <c r="BB34" t="n">
-        <v>50</v>
+      <c r="BB34" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
       <c r="BC34" t="inlineStr">
         <is>
@@ -6422,7 +6416,7 @@
         <v>50</v>
       </c>
       <c r="BI34" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="BJ34" t="n">
         <v>50</v>
@@ -6434,16 +6428,18 @@
         <v>50</v>
       </c>
       <c r="BM34" t="n">
-        <v>12150</v>
+        <v>51200</v>
       </c>
       <c r="BN34" t="n">
-        <v>12150</v>
+        <v>51200</v>
       </c>
       <c r="BO34" t="n">
-        <v>12150</v>
-      </c>
-      <c r="BP34" t="n">
-        <v>50</v>
+        <v>51200</v>
+      </c>
+      <c r="BP34" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
       <c r="BQ34" t="inlineStr">
         <is>
@@ -6461,34 +6457,40 @@
         </is>
       </c>
       <c r="BU34" t="n">
-        <v>12150</v>
+        <v>51200</v>
       </c>
       <c r="BV34" t="n">
-        <v>12150</v>
+        <v>51200</v>
       </c>
       <c r="BW34" t="n">
-        <v>12150</v>
+        <v>51200</v>
       </c>
       <c r="BX34" t="n">
-        <v>12150</v>
+        <v>51200</v>
       </c>
       <c r="BY34" t="n">
-        <v>12150</v>
+        <v>51200</v>
       </c>
       <c r="BZ34" t="n">
-        <v>12150</v>
+        <v>51200</v>
       </c>
       <c r="CA34" t="n">
-        <v>12150</v>
-      </c>
-      <c r="CB34" t="n">
-        <v>50</v>
-      </c>
-      <c r="CC34" t="n">
-        <v>50</v>
-      </c>
-      <c r="CD34" t="n">
-        <v>50</v>
+        <v>51200</v>
+      </c>
+      <c r="CB34" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="CC34" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="CD34" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
       <c r="CE34" t="inlineStr">
         <is>
@@ -6508,34 +6510,36 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>17.63</v>
+        <v>41.8</v>
       </c>
       <c r="D35" t="n">
-        <v>12.32</v>
+        <v>29.21</v>
       </c>
       <c r="E35" t="n">
-        <v>27.54</v>
+        <v>48.95</v>
       </c>
       <c r="F35" t="n">
-        <v>13.55</v>
+        <v>32.12</v>
       </c>
       <c r="G35" t="n">
         <v>1.48</v>
       </c>
       <c r="H35" t="n">
-        <v>25.3</v>
+        <v>44.98</v>
       </c>
       <c r="I35" t="n">
-        <v>2.15</v>
+        <v>2.87</v>
       </c>
       <c r="J35" t="n">
-        <v>21.26</v>
+        <v>37.8</v>
       </c>
       <c r="K35" t="n">
-        <v>1.85</v>
-      </c>
-      <c r="L35" t="n">
-        <v>0.11</v>
+        <v>2.47</v>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
       <c r="M35" t="n">
         <v>1.060827192376486</v>
@@ -6569,16 +6573,18 @@
         <v>7.91</v>
       </c>
       <c r="W35" t="n">
-        <v>83.84999999999999</v>
+        <v>149.07</v>
       </c>
       <c r="X35" t="n">
-        <v>335.53</v>
+        <v>795.34</v>
       </c>
       <c r="Y35" t="n">
-        <v>18.71</v>
-      </c>
-      <c r="Z35" t="n">
-        <v>0.04</v>
+        <v>24.95</v>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
       <c r="AA35" t="n">
         <v>1.268641495806315</v>
@@ -6594,34 +6600,40 @@
         </is>
       </c>
       <c r="AE35" t="n">
-        <v>163.99</v>
+        <v>388.71</v>
       </c>
       <c r="AF35" t="n">
-        <v>10.35</v>
+        <v>13.8</v>
       </c>
       <c r="AG35" t="n">
-        <v>15.83</v>
+        <v>28.14</v>
       </c>
       <c r="AH35" t="n">
-        <v>206.32</v>
+        <v>652.0599999999999</v>
       </c>
       <c r="AI35" t="n">
         <v>6.43</v>
       </c>
       <c r="AJ35" t="n">
-        <v>14.22</v>
+        <v>18.96</v>
       </c>
       <c r="AK35" t="n">
-        <v>46.88</v>
-      </c>
-      <c r="AL35" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="AM35" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="AN35" t="n">
-        <v>0.22</v>
+        <v>83.34</v>
+      </c>
+      <c r="AL35" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="AM35" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="AN35" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
       <c r="AO35" t="n">
         <v>1.00520894419395</v>
@@ -6637,25 +6649,25 @@
         </is>
       </c>
       <c r="AS35" t="n">
-        <v>189.99</v>
+        <v>800.63</v>
       </c>
       <c r="AT35" t="n">
-        <v>195.43</v>
+        <v>823.54</v>
       </c>
       <c r="AU35" t="n">
-        <v>160.43</v>
+        <v>676.05</v>
       </c>
       <c r="AV35" t="n">
-        <v>192.03</v>
+        <v>809.21</v>
       </c>
       <c r="AW35" t="n">
-        <v>140.59</v>
+        <v>592.4299999999999</v>
       </c>
       <c r="AX35" t="n">
-        <v>37.87</v>
+        <v>67.31999999999999</v>
       </c>
       <c r="AY35" t="n">
-        <v>4.86</v>
+        <v>6.48</v>
       </c>
       <c r="AZ35" t="n">
         <v>3.2</v>
@@ -6663,8 +6675,10 @@
       <c r="BA35" t="n">
         <v>1.84</v>
       </c>
-      <c r="BB35" t="n">
-        <v>0.08</v>
+      <c r="BB35" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
       <c r="BC35" t="n">
         <v>1.003107394252233</v>
@@ -6686,7 +6700,7 @@
         <v>4.66</v>
       </c>
       <c r="BI35" t="n">
-        <v>4.1</v>
+        <v>5.47</v>
       </c>
       <c r="BJ35" t="n">
         <v>0.86</v>
@@ -6698,16 +6712,18 @@
         <v>1.28</v>
       </c>
       <c r="BM35" t="n">
-        <v>296.78</v>
+        <v>1250.64</v>
       </c>
       <c r="BN35" t="n">
-        <v>265.69</v>
+        <v>1119.6</v>
       </c>
       <c r="BO35" t="n">
-        <v>236.73</v>
-      </c>
-      <c r="BP35" t="n">
-        <v>0.15</v>
+        <v>997.58</v>
+      </c>
+      <c r="BP35" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
       <c r="BQ35" t="n">
         <v>1.003317975839419</v>
@@ -6723,34 +6739,40 @@
         </is>
       </c>
       <c r="BU35" t="n">
-        <v>246.22</v>
+        <v>1037.58</v>
       </c>
       <c r="BV35" t="n">
-        <v>200.92</v>
+        <v>846.6900000000001</v>
       </c>
       <c r="BW35" t="n">
-        <v>146.58</v>
+        <v>617.7</v>
       </c>
       <c r="BX35" t="n">
-        <v>1134.42</v>
+        <v>4780.43</v>
       </c>
       <c r="BY35" t="n">
-        <v>684.5599999999999</v>
+        <v>2884.73</v>
       </c>
       <c r="BZ35" t="n">
-        <v>417.58</v>
+        <v>1759.68</v>
       </c>
       <c r="CA35" t="n">
-        <v>486.25</v>
-      </c>
-      <c r="CB35" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="CC35" t="n">
-        <v>0.19</v>
-      </c>
-      <c r="CD35" t="n">
-        <v>0.07000000000000001</v>
+        <v>2049.06</v>
+      </c>
+      <c r="CB35" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="CC35" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="CD35" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
       </c>
       <c r="CE35" t="n">
         <v>1.005181940612008</v>
@@ -7071,22 +7093,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>ELISA Run Parameters</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Standard Curve</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n"/>
+      <c r="B3" s="9" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Starting Concentration (ng/mL)</t>
         </is>
@@ -7096,7 +7118,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Dilution Factor</t>
         </is>
@@ -7106,7 +7128,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Dilution Series</t>
         </is>
@@ -7137,15 +7159,15 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Samples</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n"/>
+      <c r="B8" s="9" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Starting Dilution Factor</t>
         </is>
@@ -7155,17 +7177,17 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Dilution Factor</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>Dilution Series</t>
         </is>
@@ -7174,61 +7196,61 @@
         <v>50</v>
       </c>
       <c r="C11" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="D11" t="n">
-        <v>450</v>
+        <v>800</v>
       </c>
       <c r="E11" t="n">
-        <v>1350</v>
+        <v>3200</v>
       </c>
       <c r="F11" t="n">
-        <v>4050</v>
+        <v>12800</v>
       </c>
       <c r="G11" t="n">
-        <v>12150</v>
+        <v>51200</v>
       </c>
       <c r="H11" t="n">
-        <v>36450</v>
+        <v>204800</v>
       </c>
       <c r="I11" t="n">
-        <v>109350</v>
+        <v>819200</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Curve Fit Parameters (4PL)</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
-      <c r="C13" s="3" t="n"/>
-      <c r="D13" s="3" t="n"/>
+      <c r="B13" s="9" t="n"/>
+      <c r="C13" s="9" t="n"/>
+      <c r="D13" s="9" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>Parameter</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Lower Bound</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>Initial Guess</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>Upper Bound</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>Bottom</t>
         </is>
@@ -7244,7 +7266,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>Top</t>
         </is>
@@ -7260,7 +7282,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>IC50</t>
         </is>
@@ -7276,7 +7298,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>Hill</t>
         </is>
@@ -7310,14 +7332,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>SOP ELISA</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>Kasimir Reich  |  03-20-2026</t>
         </is>
@@ -7325,14 +7347,14 @@
     </row>
     <row r="3" ht="6" customHeight="1"/>
     <row r="4" ht="30" customHeight="1">
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>Goal: An enzyme-linked immunosorbent assay (ELISA) is described, which can be used to determine the quantity of antibodies or other proteins. Attached is an Excel file for calculations.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>Estimated Time: Coating usually takes &lt; 30 minutes the evening before, then around a day including waiting times.</t>
         </is>
@@ -7340,12 +7362,12 @@
     </row>
     <row r="6" ht="5" customHeight="1"/>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>PREPARATION</t>
         </is>
@@ -7353,72 +7375,72 @@
     </row>
     <row r="8" ht="4" customHeight="1"/>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>1.1</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>Planning of the Plates</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>1.</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>Determine the number and type of samples. Decide which proteins or antibodies to test for.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="56" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>2.</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>Plan the plates. Around 15 plates can be run on a single day, but start with a lower number if still gaining experience. On each plate, the first column should be a negative control with water (blank). The last should be the positive control of known concentration (standard). Each column is the dilution series for a single sample.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>3.</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>Plan the starting dilution and the dilution coefficient for both samples and standard. For example: Start with 1:50 for samples and then dilute 1:3. Start with 1000 ng/mL for the standard and do a 1:5 dilution.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>4.</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
         <is>
           <t>Do the calculations using the Excel spreadsheet.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>5.</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="14" t="inlineStr">
         <is>
           <t>Check that the washing machine is available for the day of your ELISA.</t>
         </is>
@@ -7426,7 +7448,7 @@
     </row>
     <row r="15" ht="3" customHeight="1"/>
     <row r="16" ht="11" customHeight="1">
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B16" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">· · · · · · · · · · · · · · · · · ·   Flexible Break Point  · · · · · · · · · · · · · · · · · · </t>
         </is>
@@ -7435,120 +7457,120 @@
     <row r="17" ht="3" customHeight="1"/>
     <row r="18" ht="4" customHeight="1"/>
     <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>1.2</t>
         </is>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="16" t="inlineStr">
         <is>
           <t>Coating</t>
         </is>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1">
-      <c r="A20" s="11" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>1.</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="14" t="inlineStr">
         <is>
           <t>Prepare a 2 µg/mL coating solution of the protein you want to coat with (e.g. TM4 core gp140 protein or the anti-idiotype antibody anti-3BNC117 human IgG1k). The total volume can be calculated using the spreadsheet.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>2.</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t>Prepare a wet chamber: Take the plastic box from the 4°C room. Put wet paper towels around the edges.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
-      <c r="A22" s="11" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>3.</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>Take a flat bottom ELISA 96-well plate.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>4.</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B23" s="14" t="inlineStr">
         <is>
           <t>Fill 25 µL of the coating solution into each well.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
-      <c r="A24" s="11" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>5.</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>Put the plate into the wet chamber box and put the box into the 4°C room.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
-      <c r="A25" s="11" t="inlineStr">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>6.</t>
         </is>
       </c>
-      <c r="B25" s="8" t="inlineStr">
+      <c r="B25" s="14" t="inlineStr">
         <is>
           <t>Repeat for all plates.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>7.</t>
         </is>
       </c>
-      <c r="B26" s="8" t="inlineStr">
+      <c r="B26" s="14" t="inlineStr">
         <is>
           <t>Let the plates incubate overnight.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="28" customHeight="1">
-      <c r="A27" s="11" t="inlineStr">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>8.</t>
         </is>
       </c>
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B27" s="14" t="inlineStr">
         <is>
           <t>Check whether blocking solution (5% milk) is prepared. It can be found in the door of the Mr. Shiny fridge.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="42" customHeight="1">
-      <c r="A28" s="11" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>9.</t>
         </is>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="B28" s="14" t="inlineStr">
         <is>
           <t>If not, prepare new 5% milk: Take a fresh bottle of 1X PBS (Attention: not 10X!). Go to the weighing room and add 25 g of milk powder. Mix well by inverting and put into the fridge door.</t>
         </is>
@@ -7556,7 +7578,7 @@
     </row>
     <row r="29" ht="3" customHeight="1"/>
     <row r="30" ht="11" customHeight="1">
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B30" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">· · · · · · · · · · · · · · · · · ·   Overnight Break Point  · · · · · · · · · · · · · · · · · · </t>
         </is>
@@ -7565,19 +7587,19 @@
     <row r="31" ht="3" customHeight="1"/>
     <row r="32" ht="5" customHeight="1"/>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="9" t="inlineStr">
+      <c r="A33" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B33" s="15" t="inlineStr">
         <is>
           <t>PERFORMING THE ELISA</t>
         </is>
       </c>
     </row>
     <row r="34" ht="42" customHeight="1">
-      <c r="B34" s="8" t="inlineStr">
+      <c r="B34" s="14" t="inlineStr">
         <is>
           <t>Work one plate at a time to avoid the drying out of plates. If plates dry out, the margins will have a higher signal in the measurements (edge effect). Always keep the plates covered by another (empty) plate. Keep in the wet chamber as much as possible.</t>
         </is>
@@ -7585,108 +7607,108 @@
     </row>
     <row r="35" ht="4" customHeight="1"/>
     <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="10" t="inlineStr">
+      <c r="A36" s="16" t="inlineStr">
         <is>
           <t>2.1</t>
         </is>
       </c>
-      <c r="B36" s="10" t="inlineStr">
+      <c r="B36" s="16" t="inlineStr">
         <is>
           <t>Blocking</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
-      <c r="A37" s="11" t="inlineStr">
+      <c r="A37" s="17" t="inlineStr">
         <is>
           <t>1.</t>
         </is>
       </c>
-      <c r="B37" s="8" t="inlineStr">
+      <c r="B37" s="14" t="inlineStr">
         <is>
           <t>Take the plates from the 4°C room.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
-      <c r="A38" s="11" t="inlineStr">
+      <c r="A38" s="17" t="inlineStr">
         <is>
           <t>2.</t>
         </is>
       </c>
-      <c r="B38" s="8" t="inlineStr">
+      <c r="B38" s="14" t="inlineStr">
         <is>
           <t>Throw out the coating solution and blot dry.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
-      <c r="A39" s="11" t="inlineStr">
+      <c r="A39" s="17" t="inlineStr">
         <is>
           <t>3.</t>
         </is>
       </c>
-      <c r="B39" s="8" t="inlineStr">
+      <c r="B39" s="14" t="inlineStr">
         <is>
           <t>Add 170 µL of the 5% milk to each well using the automatic multichannel pipette.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
-      <c r="A40" s="11" t="inlineStr">
+      <c r="A40" s="17" t="inlineStr">
         <is>
           <t>4.</t>
         </is>
       </c>
-      <c r="B40" s="8" t="inlineStr">
+      <c r="B40" s="14" t="inlineStr">
         <is>
           <t>Incubate for 2 h in the wet chamber at room temperature.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
-      <c r="A41" s="11" t="inlineStr">
+      <c r="A41" s="17" t="inlineStr">
         <is>
           <t>5.</t>
         </is>
       </c>
-      <c r="B41" s="8" t="inlineStr">
+      <c r="B41" s="14" t="inlineStr">
         <is>
           <t>Prepare for later steps:</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
-      <c r="A42" s="11" t="inlineStr">
+      <c r="A42" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  (a)</t>
         </is>
       </c>
-      <c r="B42" s="8" t="inlineStr">
+      <c r="B42" s="14" t="inlineStr">
         <is>
           <t>Take all samples from the freezer and let them unthaw.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="28" customHeight="1">
-      <c r="A43" s="11" t="inlineStr">
+      <c r="A43" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  (b)</t>
         </is>
       </c>
-      <c r="B43" s="8" t="inlineStr">
+      <c r="B43" s="14" t="inlineStr">
         <is>
           <t>Get the secondary antibody (Harry's ELISA box in the Mr. Shiny fridge) and the standard (freezer below Harry's bench) and keep them on ice.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="28" customHeight="1">
-      <c r="A44" s="11" t="inlineStr">
+      <c r="A44" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  (c)</t>
         </is>
       </c>
-      <c r="B44" s="8" t="inlineStr">
+      <c r="B44" s="14" t="inlineStr">
         <is>
           <t>Take the TMB solutions for the enzymatic reaction out of the 4°C room and let them warm up to room temperature.</t>
         </is>
@@ -7694,7 +7716,7 @@
     </row>
     <row r="45" ht="3" customHeight="1"/>
     <row r="46" ht="11" customHeight="1">
-      <c r="B46" s="12" t="inlineStr">
+      <c r="B46" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">· · · · · · · · · · · · · · · · · ·   Coffee Break Point  · · · · · · · · · · · · · · · · · · </t>
         </is>
@@ -7703,211 +7725,211 @@
     <row r="47" ht="3" customHeight="1"/>
     <row r="48" ht="4" customHeight="1"/>
     <row r="49" ht="16" customHeight="1">
-      <c r="A49" s="10" t="inlineStr">
+      <c r="A49" s="16" t="inlineStr">
         <is>
           <t>2.2</t>
         </is>
       </c>
-      <c r="B49" s="10" t="inlineStr">
+      <c r="B49" s="16" t="inlineStr">
         <is>
           <t>Preparation of Dilution Series and Sample Loading</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
-      <c r="B50" s="8" t="inlineStr">
+      <c r="B50" s="14" t="inlineStr">
         <is>
           <t>Once the samples are ready, start making the dilution series.</t>
         </is>
       </c>
     </row>
     <row r="51" ht="28" customHeight="1">
-      <c r="A51" s="11" t="inlineStr">
+      <c r="A51" s="17" t="inlineStr">
         <is>
           <t>1.</t>
         </is>
       </c>
-      <c r="B51" s="8" t="inlineStr">
+      <c r="B51" s="14" t="inlineStr">
         <is>
           <t>Take a V-shaped 96 ELISA well plate and begin by preparing with PBS (e.g. 120 µL into each well of the first row and 90 µL into the others).</t>
         </is>
       </c>
     </row>
     <row r="52" ht="28" customHeight="1">
-      <c r="A52" s="11" t="inlineStr">
+      <c r="A52" s="17" t="inlineStr">
         <is>
           <t>2.</t>
         </is>
       </c>
-      <c r="B52" s="8" t="inlineStr">
+      <c r="B52" s="14" t="inlineStr">
         <is>
           <t>Leave the blank and add the serum (e.g. 2.4 µL for 1:50) starting dilution for each sample into the first row.</t>
         </is>
       </c>
     </row>
     <row r="53" ht="28" customHeight="1">
-      <c r="A53" s="11" t="inlineStr">
+      <c r="A53" s="17" t="inlineStr">
         <is>
           <t>3.</t>
         </is>
       </c>
-      <c r="B53" s="8" t="inlineStr">
+      <c r="B53" s="14" t="inlineStr">
         <is>
           <t>Use the "Pipette and Mix" mode of the automatic multichannel pipette to mix and transfer (e.g. 30 µL for 1:4).</t>
         </is>
       </c>
     </row>
     <row r="54" ht="28" customHeight="1">
-      <c r="A54" s="11" t="inlineStr">
+      <c r="A54" s="17" t="inlineStr">
         <is>
           <t>4.</t>
         </is>
       </c>
-      <c r="B54" s="8" t="inlineStr">
+      <c r="B54" s="14" t="inlineStr">
         <is>
           <t>Prepare the standard once for all the plates using 8 FACS tubes (e.g. start at 1000 ng/mL in 625 µL and then transfer 125 µL to 500 µL to a 1:5 dilution).</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1">
-      <c r="A55" s="11" t="inlineStr">
+      <c r="A55" s="17" t="inlineStr">
         <is>
           <t>5.</t>
         </is>
       </c>
-      <c r="B55" s="8" t="inlineStr">
+      <c r="B55" s="14" t="inlineStr">
         <is>
           <t>Once the blocking time is passed, wash plates using the plate washer George Washington.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1">
-      <c r="A56" s="11" t="inlineStr">
+      <c r="A56" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  (a)</t>
         </is>
       </c>
-      <c r="B56" s="8" t="inlineStr">
+      <c r="B56" s="14" t="inlineStr">
         <is>
           <t>Before opening any bottle be sure to depressurize!</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
-      <c r="A57" s="11" t="inlineStr">
+      <c r="A57" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  (b)</t>
         </is>
       </c>
-      <c r="B57" s="8" t="inlineStr">
+      <c r="B57" s="14" t="inlineStr">
         <is>
           <t>Check that the PBS and water bottles are full and the trash empty.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="42" customHeight="1">
-      <c r="A58" s="11" t="inlineStr">
+      <c r="A58" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  (c)</t>
         </is>
       </c>
-      <c r="B58" s="8" t="inlineStr">
+      <c r="B58" s="14" t="inlineStr">
         <is>
           <t>Prime the machine using the yellow bottle (PBS). Sometimes there is a problem with the pressure. This can often be circumvented by having the bottle fully filled and checking the cap. Depressurize before opening.</t>
         </is>
       </c>
     </row>
     <row r="59" ht="28" customHeight="1">
-      <c r="A59" s="11" t="inlineStr">
+      <c r="A59" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  (d)</t>
         </is>
       </c>
-      <c r="B59" s="8" t="inlineStr">
+      <c r="B59" s="14" t="inlineStr">
         <is>
           <t>Load the plates into the front tower and cover both towers with empty plates to prevent the plates from drying out.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
-      <c r="A60" s="11" t="inlineStr">
+      <c r="A60" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  (e)</t>
         </is>
       </c>
-      <c r="B60" s="8" t="inlineStr">
+      <c r="B60" s="14" t="inlineStr">
         <is>
           <t>Select the program halfwell 6x PBS and click run.</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
-      <c r="A61" s="11" t="inlineStr">
+      <c r="A61" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  (f)</t>
         </is>
       </c>
-      <c r="B61" s="8" t="inlineStr">
+      <c r="B61" s="14" t="inlineStr">
         <is>
           <t>After the plates are washed, prime with water (green).</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
-      <c r="A62" s="11" t="inlineStr">
+      <c r="A62" s="17" t="inlineStr">
         <is>
           <t>6.</t>
         </is>
       </c>
-      <c r="B62" s="8" t="inlineStr">
+      <c r="B62" s="14" t="inlineStr">
         <is>
           <t>Load 25 µL of the samples:</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
-      <c r="A63" s="11" t="inlineStr">
+      <c r="A63" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  (a)</t>
         </is>
       </c>
-      <c r="B63" s="8" t="inlineStr">
+      <c r="B63" s="14" t="inlineStr">
         <is>
           <t>Throw out the washing PBS and blot dry.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="42" customHeight="1">
-      <c r="A64" s="11" t="inlineStr">
+      <c r="A64" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  (b)</t>
         </is>
       </c>
-      <c r="B64" s="8" t="inlineStr">
+      <c r="B64" s="14" t="inlineStr">
         <is>
           <t>Using a normal multichannel transfer 25 µL of the dilution series: Reuse the tips. Start with the highest dilution, transfer without blowing out, blow out over the original dilution and then move on to the next highest dilution.</t>
         </is>
       </c>
     </row>
     <row r="65" ht="28" customHeight="1">
-      <c r="A65" s="11" t="inlineStr">
+      <c r="A65" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  (c)</t>
         </is>
       </c>
-      <c r="B65" s="8" t="inlineStr">
+      <c r="B65" s="14" t="inlineStr">
         <is>
           <t>To keep things simple, use a second pipette to transfer the standard and reuse these tips.</t>
         </is>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1">
-      <c r="A66" s="11" t="inlineStr">
+      <c r="A66" s="17" t="inlineStr">
         <is>
           <t>7.</t>
         </is>
       </c>
-      <c r="B66" s="8" t="inlineStr">
+      <c r="B66" s="14" t="inlineStr">
         <is>
           <t>Incubate for 1.5 h in the wet chamber at room temperature.</t>
         </is>
@@ -7915,7 +7937,7 @@
     </row>
     <row r="67" ht="3" customHeight="1"/>
     <row r="68" ht="11" customHeight="1">
-      <c r="B68" s="12" t="inlineStr">
+      <c r="B68" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">· · · · · · · · · · · · · · · · · ·   Lunch Break Point  · · · · · · · · · · · · · · · · · · </t>
         </is>
@@ -7924,72 +7946,72 @@
     <row r="69" ht="3" customHeight="1"/>
     <row r="70" ht="4" customHeight="1"/>
     <row r="71" ht="16" customHeight="1">
-      <c r="A71" s="10" t="inlineStr">
+      <c r="A71" s="16" t="inlineStr">
         <is>
           <t>2.3</t>
         </is>
       </c>
-      <c r="B71" s="10" t="inlineStr">
+      <c r="B71" s="16" t="inlineStr">
         <is>
           <t>Adding the Secondary Antibody</t>
         </is>
       </c>
     </row>
     <row r="72" ht="28" customHeight="1">
-      <c r="A72" s="11" t="inlineStr">
+      <c r="A72" s="17" t="inlineStr">
         <is>
           <t>1.</t>
         </is>
       </c>
-      <c r="B72" s="8" t="inlineStr">
+      <c r="B72" s="14" t="inlineStr">
         <is>
           <t>After incubation, wash the plates using the program halfwell 6x PBS. Prime with PBS before and with water after.</t>
         </is>
       </c>
     </row>
     <row r="73" ht="42" customHeight="1">
-      <c r="A73" s="11" t="inlineStr">
+      <c r="A73" s="17" t="inlineStr">
         <is>
           <t>2.</t>
         </is>
       </c>
-      <c r="B73" s="8" t="inlineStr">
+      <c r="B73" s="14" t="inlineStr">
         <is>
           <t>Meanwhile, prepare a 1:5000 dilution of the secondary antibody (e.g. anti-mouse IgG-HRP, antibody is Jackson Cat. 115-035-071 (0.8 mg/mL Harry April 2025)). Calculate the needed volume using the table. (25 µL × 96 wells × plate number + a little extra)</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1">
-      <c r="A74" s="11" t="inlineStr">
+      <c r="A74" s="17" t="inlineStr">
         <is>
           <t>3.</t>
         </is>
       </c>
-      <c r="B74" s="8" t="inlineStr">
+      <c r="B74" s="14" t="inlineStr">
         <is>
           <t>Throw away the washing PBS and blot dry.</t>
         </is>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1">
-      <c r="A75" s="11" t="inlineStr">
+      <c r="A75" s="17" t="inlineStr">
         <is>
           <t>4.</t>
         </is>
       </c>
-      <c r="B75" s="8" t="inlineStr">
+      <c r="B75" s="14" t="inlineStr">
         <is>
           <t>Add 25 µL of the secondary antibody solution.</t>
         </is>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1">
-      <c r="A76" s="11" t="inlineStr">
+      <c r="A76" s="17" t="inlineStr">
         <is>
           <t>5.</t>
         </is>
       </c>
-      <c r="B76" s="8" t="inlineStr">
+      <c r="B76" s="14" t="inlineStr">
         <is>
           <t>Incubate for 1 h in the wet chamber at room temperature.</t>
         </is>
@@ -7997,7 +8019,7 @@
     </row>
     <row r="77" ht="3" customHeight="1"/>
     <row r="78" ht="11" customHeight="1">
-      <c r="B78" s="12" t="inlineStr">
+      <c r="B78" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">· · · · · · · · · · · · · · · · · ·   Coffee Break Point  · · · · · · · · · · · · · · · · · · </t>
         </is>
@@ -8006,96 +8028,96 @@
     <row r="79" ht="3" customHeight="1"/>
     <row r="80" ht="4" customHeight="1"/>
     <row r="81" ht="16" customHeight="1">
-      <c r="A81" s="10" t="inlineStr">
+      <c r="A81" s="16" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="B81" s="10" t="inlineStr">
+      <c r="B81" s="16" t="inlineStr">
         <is>
           <t>Performing the Enzymatic Reaction</t>
         </is>
       </c>
     </row>
     <row r="82" ht="42" customHeight="1">
-      <c r="A82" s="11" t="inlineStr">
+      <c r="A82" s="17" t="inlineStr">
         <is>
           <t>1.</t>
         </is>
       </c>
-      <c r="B82" s="8" t="inlineStr">
+      <c r="B82" s="14" t="inlineStr">
         <is>
           <t>After incubation, wash the plates using the program halfwell 6x PBS. Prime with PBS before and with water after. If you're likely to be the last person using the machine that day, start the shut down sequence — this cleans and depressurizes the machine.</t>
         </is>
       </c>
     </row>
     <row r="83" ht="28" customHeight="1">
-      <c r="A83" s="11" t="inlineStr">
+      <c r="A83" s="17" t="inlineStr">
         <is>
           <t>2.</t>
         </is>
       </c>
-      <c r="B83" s="8" t="inlineStr">
+      <c r="B83" s="14" t="inlineStr">
         <is>
           <t>Meanwhile, prepare a 1:1 mix of the TMB substrate and the H₂O₂. In total, it's double the volume of the secondary antibody stain.</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1">
-      <c r="A84" s="11" t="inlineStr">
+      <c r="A84" s="17" t="inlineStr">
         <is>
           <t>3.</t>
         </is>
       </c>
-      <c r="B84" s="8" t="inlineStr">
+      <c r="B84" s="14" t="inlineStr">
         <is>
           <t>Throw away the washing PBS and blot dry.</t>
         </is>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1">
-      <c r="A85" s="11" t="inlineStr">
+      <c r="A85" s="17" t="inlineStr">
         <is>
           <t>4.</t>
         </is>
       </c>
-      <c r="B85" s="8" t="inlineStr">
+      <c r="B85" s="14" t="inlineStr">
         <is>
           <t>Add 50 µL of the solution to each well.</t>
         </is>
       </c>
     </row>
     <row r="86" ht="28" customHeight="1">
-      <c r="A86" s="11" t="inlineStr">
+      <c r="A86" s="17" t="inlineStr">
         <is>
           <t>5.</t>
         </is>
       </c>
-      <c r="B86" s="8" t="inlineStr">
+      <c r="B86" s="14" t="inlineStr">
         <is>
           <t>Develop the reaction for around 12 min until the highest concentration of standard is maxed out.</t>
         </is>
       </c>
     </row>
     <row r="87" ht="28" customHeight="1">
-      <c r="A87" s="11" t="inlineStr">
+      <c r="A87" s="17" t="inlineStr">
         <is>
           <t>6.</t>
         </is>
       </c>
-      <c r="B87" s="8" t="inlineStr">
+      <c r="B87" s="14" t="inlineStr">
         <is>
           <t>Stop the reaction using 50 µL of 1 M H₂SO₄. Attention: Do not let any H₂SO₄ come on your clothes or skin!</t>
         </is>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1">
-      <c r="A88" s="11" t="inlineStr">
+      <c r="A88" s="17" t="inlineStr">
         <is>
           <t>7.</t>
         </is>
       </c>
-      <c r="B88" s="8" t="inlineStr">
+      <c r="B88" s="14" t="inlineStr">
         <is>
           <t>Read immediately afterwards using the plate reader.</t>
         </is>
@@ -8103,84 +8125,84 @@
     </row>
     <row r="89" ht="4" customHeight="1"/>
     <row r="90" ht="16" customHeight="1">
-      <c r="A90" s="10" t="inlineStr">
+      <c r="A90" s="16" t="inlineStr">
         <is>
           <t>2.5</t>
         </is>
       </c>
-      <c r="B90" s="10" t="inlineStr">
+      <c r="B90" s="16" t="inlineStr">
         <is>
           <t>Reading the Results</t>
         </is>
       </c>
     </row>
     <row r="91" ht="42" customHeight="1">
-      <c r="A91" s="11" t="inlineStr">
+      <c r="A91" s="17" t="inlineStr">
         <is>
           <t>1.</t>
         </is>
       </c>
-      <c r="B91" s="8" t="inlineStr">
+      <c r="B91" s="14" t="inlineStr">
         <is>
           <t>Use the plate reader machine. Open the Omega software and use the experiment Harry 450 and 570. 450 nm is the wavelength of the reaction. 570 nm is for measuring potential contamination or dirt.</t>
         </is>
       </c>
     </row>
     <row r="92" ht="15" customHeight="1">
-      <c r="A92" s="11" t="inlineStr">
+      <c r="A92" s="17" t="inlineStr">
         <is>
           <t>2.</t>
         </is>
       </c>
-      <c r="B92" s="8" t="inlineStr">
+      <c r="B92" s="14" t="inlineStr">
         <is>
           <t>Name the plates with date, experiment name, and number.</t>
         </is>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1">
-      <c r="A93" s="11" t="inlineStr">
+      <c r="A93" s="17" t="inlineStr">
         <is>
           <t>3.</t>
         </is>
       </c>
-      <c r="B93" s="8" t="inlineStr">
+      <c r="B93" s="14" t="inlineStr">
         <is>
           <t>Use the software to open the plate holder and insert the plate.</t>
         </is>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1">
-      <c r="A94" s="11" t="inlineStr">
+      <c r="A94" s="17" t="inlineStr">
         <is>
           <t>4.</t>
         </is>
       </c>
-      <c r="B94" s="8" t="inlineStr">
+      <c r="B94" s="14" t="inlineStr">
         <is>
           <t>Start an experiment.</t>
         </is>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1">
-      <c r="A95" s="11" t="inlineStr">
+      <c r="A95" s="17" t="inlineStr">
         <is>
           <t>5.</t>
         </is>
       </c>
-      <c r="B95" s="8" t="inlineStr">
+      <c r="B95" s="14" t="inlineStr">
         <is>
           <t>Wait... (Great time to talk to someone or do some flashcards.)</t>
         </is>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1">
-      <c r="A96" s="11" t="inlineStr">
+      <c r="A96" s="17" t="inlineStr">
         <is>
           <t>6.</t>
         </is>
       </c>
-      <c r="B96" s="8" t="inlineStr">
+      <c r="B96" s="14" t="inlineStr">
         <is>
           <t>Repeat for all plates.</t>
         </is>
@@ -8188,48 +8210,48 @@
     </row>
     <row r="97" ht="4" customHeight="1"/>
     <row r="98" ht="16" customHeight="1">
-      <c r="A98" s="10" t="inlineStr">
+      <c r="A98" s="16" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="B98" s="10" t="inlineStr">
+      <c r="B98" s="16" t="inlineStr">
         <is>
           <t>Transfer of Data</t>
         </is>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1">
-      <c r="A99" s="11" t="inlineStr">
+      <c r="A99" s="17" t="inlineStr">
         <is>
           <t>1.</t>
         </is>
       </c>
-      <c r="B99" s="8" t="inlineStr">
+      <c r="B99" s="14" t="inlineStr">
         <is>
           <t>Open the Omega Analysis Software.</t>
         </is>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1">
-      <c r="A100" s="11" t="inlineStr">
+      <c r="A100" s="17" t="inlineStr">
         <is>
           <t>2.</t>
         </is>
       </c>
-      <c r="B100" s="8" t="inlineStr">
+      <c r="B100" s="14" t="inlineStr">
         <is>
           <t>Click on open, select all the files and right-click them to select "Export as multiple ASCII files".</t>
         </is>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1">
-      <c r="A101" s="11" t="inlineStr">
+      <c r="A101" s="17" t="inlineStr">
         <is>
           <t>3.</t>
         </is>
       </c>
-      <c r="B101" s="8" t="inlineStr">
+      <c r="B101" s="14" t="inlineStr">
         <is>
           <t>Save the data to the folder "tempshare/*yourname*".</t>
         </is>
@@ -8237,7 +8259,7 @@
     </row>
     <row r="102" ht="3" customHeight="1"/>
     <row r="103" ht="11" customHeight="1">
-      <c r="B103" s="12" t="inlineStr">
+      <c r="B103" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">· · · · · · · · · · · · · · · · · ·   Flexible Break Point  · · · · · · · · · · · · · · · · · · </t>
         </is>
@@ -8246,12 +8268,12 @@
     <row r="104" ht="3" customHeight="1"/>
     <row r="105" ht="5" customHeight="1"/>
     <row r="106" ht="18" customHeight="1">
-      <c r="A106" s="9" t="inlineStr">
+      <c r="A106" s="15" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B106" s="9" t="inlineStr">
+      <c r="B106" s="15" t="inlineStr">
         <is>
           <t>ANALYSIS</t>
         </is>
@@ -8259,60 +8281,60 @@
     </row>
     <row r="107" ht="4" customHeight="1"/>
     <row r="108" ht="16" customHeight="1">
-      <c r="A108" s="10" t="inlineStr">
+      <c r="A108" s="16" t="inlineStr">
         <is>
           <t>3.1</t>
         </is>
       </c>
-      <c r="B108" s="10" t="inlineStr">
+      <c r="B108" s="16" t="inlineStr">
         <is>
           <t>Cleaning of the Data</t>
         </is>
       </c>
     </row>
     <row r="109" ht="15" customHeight="1">
-      <c r="A109" s="11" t="inlineStr">
+      <c r="A109" s="17" t="inlineStr">
         <is>
           <t>1.</t>
         </is>
       </c>
-      <c r="B109" s="8" t="inlineStr">
+      <c r="B109" s="14" t="inlineStr">
         <is>
           <t>Copy the files from tempshare to your computer.</t>
         </is>
       </c>
     </row>
     <row r="110" ht="15" customHeight="1">
-      <c r="A110" s="11" t="inlineStr">
+      <c r="A110" s="17" t="inlineStr">
         <is>
           <t>2.</t>
         </is>
       </c>
-      <c r="B110" s="8" t="inlineStr">
+      <c r="B110" s="14" t="inlineStr">
         <is>
           <t>Merge the separate files manually or using Python.</t>
         </is>
       </c>
     </row>
     <row r="111" ht="28" customHeight="1">
-      <c r="A111" s="11" t="inlineStr">
+      <c r="A111" s="17" t="inlineStr">
         <is>
           <t>3.</t>
         </is>
       </c>
-      <c r="B111" s="8" t="inlineStr">
+      <c r="B111" s="14" t="inlineStr">
         <is>
           <t>Color the individual tables according to Harry's color scheme (Red = larger) manually or using Python.</t>
         </is>
       </c>
     </row>
     <row r="112" ht="15" customHeight="1">
-      <c r="A112" s="11" t="inlineStr">
+      <c r="A112" s="17" t="inlineStr">
         <is>
           <t>4.</t>
         </is>
       </c>
-      <c r="B112" s="8" t="inlineStr">
+      <c r="B112" s="14" t="inlineStr">
         <is>
           <t>Add the sample names using Python or manually.</t>
         </is>
@@ -8320,48 +8342,48 @@
     </row>
     <row r="113" ht="4" customHeight="1"/>
     <row r="114" ht="16" customHeight="1">
-      <c r="A114" s="10" t="inlineStr">
+      <c r="A114" s="16" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="B114" s="10" t="inlineStr">
+      <c r="B114" s="16" t="inlineStr">
         <is>
           <t>Determination of EC₅₀ or Concentration</t>
         </is>
       </c>
     </row>
     <row r="115" ht="56" customHeight="1">
-      <c r="A115" s="11" t="inlineStr">
+      <c r="A115" s="17" t="inlineStr">
         <is>
           <t>1.</t>
         </is>
       </c>
-      <c r="B115" s="8" t="inlineStr">
+      <c r="B115" s="14" t="inlineStr">
         <is>
           <t>The EC₅₀ is the concentration at which half the maximum reaction occurs. It is the turning point of a sigmoidal function fitted to the data. This has the advantage of being independent of the starting concentration (as long as the data points allow for the fitting of a curve).</t>
         </is>
       </c>
     </row>
     <row r="116" ht="15" customHeight="1">
-      <c r="A116" s="11" t="inlineStr">
+      <c r="A116" s="17" t="inlineStr">
         <is>
           <t>2.</t>
         </is>
       </c>
-      <c r="B116" s="8" t="inlineStr">
+      <c r="B116" s="14" t="inlineStr">
         <is>
           <t>It can be calculated using a Prism sheet or using Python.</t>
         </is>
       </c>
     </row>
     <row r="117" ht="42" customHeight="1">
-      <c r="A117" s="11" t="inlineStr">
+      <c r="A117" s="17" t="inlineStr">
         <is>
           <t>3.</t>
         </is>
       </c>
-      <c r="B117" s="8" t="inlineStr">
+      <c r="B117" s="14" t="inlineStr">
         <is>
           <t>Based on the standard, an absolute concentration can also be calculated. This is done by fitting a function to the standard with the known concentration as x values and then using the inverse function to calculate the concentrations in the samples. Use Prism or Python.</t>
         </is>

</xml_diff>